<commit_message>
add TIDA-010954 Reference material
</commit_message>
<xml_diff>
--- a/Document/PersonalStudyMaterial/MicroInverterStuday.xlsx
+++ b/Document/PersonalStudyMaterial/MicroInverterStuday.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\micinvertergit\micinveter\Document\PersonalStudyMaterial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D74AB27-3C19-4B72-BFA7-E42C0409AEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3DC578-BB33-49D7-AA0F-AD85D8D1A660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="零馈电" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>1.外接 CT 电流互感器（阳台储能零馈电 / 防逆流),无线通信引入延迟，200‑400ms；干扰环境丢包风险；固件需要做通信容错。</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>CT 输出 → 二阶 / 四阶高通滤波（30kHz HPF，滤除 DC 与 PWM 基波）→ 运放可编程增益放大 → 高速 ADC（≥200kSPS）送入 MCU/DSP</t>
+  </si>
+  <si>
+    <t>Reference Material</t>
   </si>
 </sst>
 </file>
@@ -154,6 +157,147 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>28576</xdr:colOff>
+          <xdr:row>10</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>590550</xdr:colOff>
+          <xdr:row>17</xdr:row>
+          <xdr:rowOff>10083</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1027" name="Object 3" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1027"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E664B0D-350A-BAB3-DE3C-67844AAE4F79}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd type="none" w="med" len="med"/>
+            </a:ln>
+            <a:effectLst/>
+            <a:extLst>
+              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
+                <a14:hiddenEffects>
+                  <a:effectLst>
+                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="808080"/>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </a14:hiddenEffects>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>590549</xdr:colOff>
+          <xdr:row>9</xdr:row>
+          <xdr:rowOff>190499</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>600075</xdr:colOff>
+          <xdr:row>17</xdr:row>
+          <xdr:rowOff>2380</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1029" name="Object 5" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1029"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55C4C37B-F8C0-8A74-7DCF-1F63DB0B6AF2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd type="none" w="med" len="med"/>
+            </a:ln>
+            <a:effectLst/>
+            <a:extLst>
+              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
+                <a14:hiddenEffects>
+                  <a:effectLst>
+                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="808080"/>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </a14:hiddenEffects>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -444,35 +588,100 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDC317D-541B-4328-91ED-36C03FF8439C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="75.7109375" customWidth="1"/>
+  </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8DB093B-6028-45E0-942C-3A039F1FF350}">
-  <dimension ref="A1:A5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8DB093B-6028-45E0-942C-3A039F1FF350}">
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <oleObjects>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Acrobat Document" shapeId="1027" r:id="rId4">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId5">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>28575</xdr:colOff>
+                <xdr:row>10</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>590550</xdr:colOff>
+                <xdr:row>17</xdr:row>
+                <xdr:rowOff>9525</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Acrobat Document" shapeId="1027" r:id="rId4"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Acrobat Document" dvAspect="DVASPECT_ICON" shapeId="1029" r:id="rId6">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId7">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>590550</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>190500</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>600075</xdr:colOff>
+                <xdr:row>17</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Acrobat Document" dvAspect="DVASPECT_ICON" shapeId="1029" r:id="rId6"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </oleObjects>
 </worksheet>
 </file>
</xml_diff>